<commit_message>
Fix sticky nav on homepage, correct FAQ link consistency across site
</commit_message>
<xml_diff>
--- a/sendcleared-outreach-tracker.xlsx
+++ b/sendcleared-outreach-tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/timothyarmstead/Sendcleared/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE8B207A-B42F-9746-893D-810316C03EA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86844F5E-9339-5946-9B12-A4546D95B2EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3320" yWindow="600" windowWidth="27860" windowHeight="16220" tabRatio="500" firstSheet="3" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8980" yWindow="1740" windowWidth="27860" windowHeight="16220" tabRatio="500" firstSheet="3" activeTab="11" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="12" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1363" uniqueCount="850">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1401" uniqueCount="868">
   <si>
     <t>SendCleared — Daily Outreach Playbook  |  1 Hour / Day</t>
   </si>
@@ -2660,6 +2660,130 @@
   </si>
   <si>
     <t>15.09.26</t>
+  </si>
+  <si>
+    <t>"What is the worst email marketing mistake you've ever made or seen?"</t>
+  </si>
+  <si>
+    <r>
+      <t>"How do you prevent sending an email with broken links or bad merge tags (</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+        <family val="2"/>
+      </rPr>
+      <t>{{first_name}}</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>)?"</t>
+    </r>
+  </si>
+  <si>
+    <t>"Why do my HTML emails look broken in Outlook or Apple Mail?"</t>
+  </si>
+  <si>
+    <t>Pre-Send Process &amp; Checklists</t>
+  </si>
+  <si>
+    <t>"What is your pre-launch checklist before hitting 'Send' on an email campaign?"</t>
+  </si>
+  <si>
+    <t>"How do email marketers perform QA on automated lifecycle flows (Klaviyo, HubSpot, etc.)?"</t>
+  </si>
+  <si>
+    <t>"What is the best way to double-check email render and formatting across different clients?"</t>
+  </si>
+  <si>
+    <t>Tooling &amp; Alternatives</t>
+  </si>
+  <si>
+    <t>"Are there any good alternative tools to Litmus or Email on Acid for email QA testing?"</t>
+  </si>
+  <si>
+    <t>"What are the best automated tools to catch email bugs before broadcast?"</t>
+  </si>
+  <si>
+    <t>"How do you test dark mode rendering for HTML email newsletters?"</t>
+  </si>
+  <si>
+    <t>Strategy to Plug SendCleared on Quora</t>
+  </si>
+  <si>
+    <r>
+      <t>Provide a High-Value Framework First:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Don't just post a sales link. Give a structured 4-point manual checklist (e.g., checking subject lines/preheaders, testing live fallback tags, rendering on mobile/dark mode, verifying preview texts).</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Introduce the "Automated Solution":</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Explain that doing manual checks across every broadcast or automation update takes 15–20 minutes and still leaves room for human error.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Soft Pitch:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t>"To speed this up and catch things like broken dynamic tags or broken layouts automatically, tools like SendCleared run these pre-flight checks instantly before you send."</t>
+    </r>
+  </si>
+  <si>
+    <t>Common QA Failures &amp; Disaster Stories - Quora - Target email marketing category - will need to keep broad</t>
+  </si>
+  <si>
+    <t>Second Send</t>
+  </si>
+  <si>
+    <t>16.09.26</t>
   </si>
 </sst>
 </file>
@@ -2670,7 +2794,7 @@
     <numFmt numFmtId="164" formatCode="dd\ mmm\ yy"/>
     <numFmt numFmtId="165" formatCode="dd\ mmm\ yyyy"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2805,6 +2929,29 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="10">
     <fill>
@@ -2889,7 +3036,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2975,6 +3122,8 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5286,7 +5435,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C59208D-E153-D94F-949B-1D2F26D7FF23}">
-  <dimension ref="A1:I202"/>
+  <dimension ref="A1:J202"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="58" customWidth="1"/>
@@ -5316,6 +5465,9 @@
       <c r="F1" s="20" t="s">
         <v>553</v>
       </c>
+      <c r="G1" s="20" t="s">
+        <v>866</v>
+      </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -5346,6 +5498,9 @@
       <c r="E3" t="s">
         <v>554</v>
       </c>
+      <c r="G3" t="s">
+        <v>867</v>
+      </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
@@ -5372,6 +5527,9 @@
       <c r="E5" t="s">
         <v>554</v>
       </c>
+      <c r="G5" t="s">
+        <v>867</v>
+      </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
@@ -5387,6 +5545,9 @@
       <c r="E6" t="s">
         <v>554</v>
       </c>
+      <c r="G6" t="s">
+        <v>867</v>
+      </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -5401,6 +5562,9 @@
       <c r="E7" t="s">
         <v>554</v>
       </c>
+      <c r="G7" t="s">
+        <v>867</v>
+      </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -5415,6 +5579,9 @@
       <c r="E8" t="s">
         <v>554</v>
       </c>
+      <c r="G8" t="s">
+        <v>867</v>
+      </c>
       <c r="H8" t="s">
         <v>476</v>
       </c>
@@ -5433,6 +5600,9 @@
       <c r="E9" t="s">
         <v>554</v>
       </c>
+      <c r="G9" t="s">
+        <v>867</v>
+      </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
@@ -5460,6 +5630,9 @@
       <c r="F11" t="s">
         <v>554</v>
       </c>
+      <c r="G11" t="s">
+        <v>867</v>
+      </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -5475,6 +5648,9 @@
       <c r="F12" t="s">
         <v>554</v>
       </c>
+      <c r="G12" t="s">
+        <v>867</v>
+      </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
@@ -5490,6 +5666,9 @@
       <c r="E13" t="s">
         <v>554</v>
       </c>
+      <c r="G13" t="s">
+        <v>867</v>
+      </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
@@ -5505,6 +5684,9 @@
       <c r="E14" t="s">
         <v>554</v>
       </c>
+      <c r="G14" t="s">
+        <v>867</v>
+      </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -5535,8 +5717,11 @@
       <c r="E16" t="s">
         <v>554</v>
       </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G16" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>324</v>
       </c>
@@ -5550,8 +5735,11 @@
       <c r="E17" t="s">
         <v>554</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G17" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>455</v>
       </c>
@@ -5565,8 +5753,14 @@
       <c r="F18" t="s">
         <v>554</v>
       </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G18" t="s">
+        <v>867</v>
+      </c>
+      <c r="J18" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>300</v>
       </c>
@@ -5580,8 +5774,11 @@
       <c r="E19" t="s">
         <v>554</v>
       </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G19" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>332</v>
       </c>
@@ -5595,11 +5792,14 @@
       <c r="E20" t="s">
         <v>554</v>
       </c>
+      <c r="G20" t="s">
+        <v>867</v>
+      </c>
       <c r="I20" t="s">
         <v>476</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>303</v>
       </c>
@@ -5613,8 +5813,11 @@
       <c r="E21" t="s">
         <v>554</v>
       </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G21" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>446</v>
       </c>
@@ -5629,7 +5832,7 @@
         <v>554</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>328</v>
       </c>
@@ -5643,8 +5846,11 @@
       <c r="E23" t="s">
         <v>554</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G23" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>350</v>
       </c>
@@ -5658,8 +5864,11 @@
       <c r="E24" t="s">
         <v>554</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G24" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>474</v>
       </c>
@@ -5673,8 +5882,11 @@
       <c r="E25" t="s">
         <v>554</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G25" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>348</v>
       </c>
@@ -5686,7 +5898,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>447</v>
       </c>
@@ -5700,8 +5912,11 @@
       <c r="E27" t="s">
         <v>554</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="G27" t="s">
+        <v>867</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>468</v>
       </c>
@@ -5716,7 +5931,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>343</v>
       </c>
@@ -5731,7 +5946,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>472</v>
       </c>
@@ -5746,7 +5961,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>478</v>
       </c>
@@ -5761,7 +5976,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>323</v>
       </c>
@@ -12294,7 +12509,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
@@ -12363,6 +12578,86 @@
       </c>
       <c r="C8" s="6"/>
     </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="43" t="s">
+        <v>865</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="44" t="s">
+        <v>850</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="16" x14ac:dyDescent="0.25">
+      <c r="A14" s="44" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" s="44" t="s">
+        <v>852</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="43" t="s">
+        <v>853</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="44" t="s">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" s="44" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="44" t="s">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="43" t="s">
+        <v>857</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="44" t="s">
+        <v>858</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="44" t="s">
+        <v>859</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" s="44" t="s">
+        <v>860</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" s="43" t="s">
+        <v>861</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A36" s="43" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A38" s="43" t="s">
+        <v>863</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A40" s="43" t="s">
+        <v>864</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:C1"/>

</xml_diff>